<commit_message>
docs: arquitectura consolidada (As-Is/To-Be/Hub), estimacion de costos ampliada y Product Definition de AutoWAR
Diagrama .drawio unico de 3 paginas; costos con staging, desarrollo, Kiro y resumen financiero; documento Word de definicion de producto con analisis financiero y comercializacion; diagramas previos archivados.
</commit_message>
<xml_diff>
--- a/docs/gfourmis-sesion-arquitectura/AutoWAR-Estimacion-Costos.xlsx
+++ b/docs/gfourmis-sesion-arquitectura/AutoWAR-Estimacion-Costos.xlsx
@@ -13,6 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa Bedrock" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidad" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verif. Calculadora AWS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambientes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inversion y OPEX" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Financiero" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,10 +24,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,34 +40,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <sz val="9"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <sz val="9"/>
+      <i val="1"/>
+      <color rgb="00B85450"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -70,12 +59,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
     <fill>
@@ -85,22 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -130,76 +104,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,16 +491,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>AutoWAR - Supuestos de costo (celdas AMARILLAS = editables)</t>
@@ -584,7 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Region: us-east-1 | Moneda: USD | Precios de referencia publicos (oct-2026). Validar en la calculadora AWS para cotizacion formal.</t>
+          <t>Region: us-east-1 | Moneda: USD | Precios de referencia publicos (oct-2026). Incluye componentes To-Be (WAF, Cognito, Lambda Authorizer, entitlements). Validar en la calculadora AWS para cotizacion formal.</t>
         </is>
       </c>
     </row>
@@ -594,24 +520,24 @@
           <t>PRECIOS UNITARIOS AWS</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Fuente / nota</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Lambda: precio por request</t>
         </is>
@@ -619,19 +545,19 @@
       <c r="B5" s="5" t="n">
         <v>2e-07</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>USD/request</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>US$0.20 por 1M requests</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Lambda: precio por GB-segundo (x86)</t>
         </is>
@@ -639,19 +565,19 @@
       <c r="B6" s="5" t="n">
         <v>1.66667e-05</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>USD/GB-s</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>x86 on-demand</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Step Functions: por transicion (Standard)</t>
         </is>
@@ -659,19 +585,19 @@
       <c r="B7" s="5" t="n">
         <v>2.5e-05</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>USD/transicion</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>US$0.025 por 1.000 transiciones</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>API Gateway REST: por request</t>
         </is>
@@ -679,19 +605,19 @@
       <c r="B8" s="5" t="n">
         <v>3.5e-06</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>USD/request</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>US$3.50 por 1M requests</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>DynamoDB on-demand: por escritura (WRU)</t>
         </is>
@@ -699,19 +625,19 @@
       <c r="B9" s="5" t="n">
         <v>1.25e-06</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>USD/escritura</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>US$1.25 por 1M WRU</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>DynamoDB on-demand: por lectura (RRU)</t>
         </is>
@@ -719,19 +645,19 @@
       <c r="B10" s="5" t="n">
         <v>2.5e-07</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>USD/lectura</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>US$0.25 por 1M RRU</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>S3: almacenamiento por GB-mes</t>
         </is>
@@ -739,19 +665,19 @@
       <c r="B11" s="5" t="n">
         <v>0.023</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>USD/GB-mes</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>S3 Standard</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>CloudWatch: por GB de logs ingeridos</t>
         </is>
@@ -759,39 +685,39 @@
       <c r="B12" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>USD/GB</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>ingestion de logs</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>KMS: por clave-mes</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>USD/clave-mes</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>clave gestionada</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Secrets Manager: por secreto-mes</t>
         </is>
@@ -799,19 +725,19 @@
       <c r="B14" s="5" t="n">
         <v>0.4</v>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>USD/secreto-mes</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>+US$0.05 por 10k llamadas (despreciable)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Bedrock Sonnet: por token entrada</t>
         </is>
@@ -819,19 +745,19 @@
       <c r="B15" s="5" t="n">
         <v>3e-06</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>US$3 por 1M tokens in</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Bedrock Sonnet: por token salida</t>
         </is>
@@ -839,19 +765,19 @@
       <c r="B16" s="5" t="n">
         <v>1.5e-05</v>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>US$15 por 1M tokens out</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Bedrock Haiku: por token entrada</t>
         </is>
@@ -859,19 +785,19 @@
       <c r="B17" s="5" t="n">
         <v>8e-07</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>~US$0.80 por 1M tokens in</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Bedrock Haiku: por token salida</t>
         </is>
@@ -879,318 +805,432 @@
       <c r="B18" s="5" t="n">
         <v>4e-06</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>~US$4 por 1M tokens out</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WAF: por web ACL-mes</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>USD/web ACL-mes</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>US$5 por web ACL/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WAF: por regla/grupo-mes</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>USD/regla-mes</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>US$1 por regla o managed rule group/mes</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WAF: por millon de requests</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>USD/millon req</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>US$0.60 por 1M requests inspeccionados</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cognito: por MAU (sobre capa gratis)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>USD/MAU</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Essentials ~US$0.015/MAU; 10k MAU gratis (fed. menor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>PARAMETROS POR ANALISIS (1 cuenta, 6 pilares)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Invocaciones Lambda por analisis</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="B25" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>invocaciones</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>6 pilares + 1 orquestador</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>6 pilares + orquestador + authorizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Duracion promedio por Lambda</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B26" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>segundos</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>editable segun cuenta</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Memoria Lambda</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B27" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>1024 MB</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Transiciones Step Functions</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n">
+      <c r="B28" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>transiciones</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>fan-out + joins</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Requests API Gateway</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B29" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>requests</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>validar + analizar + polling</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Escrituras DynamoDB</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="B30" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>escrituras</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>resultados + items por pilar</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>resultados + items por pilar + entitlements</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Lecturas DynamoDB</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="B31" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>lecturas</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>lectura de resultados</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>resultados + lectura de entitlements</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Logs generados</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B32" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>~50 MB de logs por analisis</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Tokens entrada Bedrock</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B33" s="5" t="n">
         <v>15000</v>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>tokens</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>hallazgos + contexto</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Tokens salida Bedrock</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B34" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>tokens</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>resumen redactado</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>ESCENARIO MENSUAL</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Analisis por mes</t>
         </is>
       </c>
-      <c r="B35" s="8" t="n">
+      <c r="B37" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Modelo Bedrock (1=Sonnet, 2=Haiku)</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B38" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Secretos (clientes) almacenados</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n">
+      <c r="B39" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Claves KMS</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n">
+      <c r="B40" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Hosting CloudFront+S3 (fijo/mes)</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n">
+      <c r="B41" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>WAF: web ACLs</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>WAF: reglas/grupos</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>WAF: requests/mes (millones)</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Cognito: MAU facturables (sobre capa gratis)</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Entitlements: items DynamoDB (clientes activos)</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1201,15 +1241,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Costo variable por 1 analisis (1 cuenta, 6 pilares)</t>
@@ -1217,183 +1257,195 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Servicio</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Formula (de donde sale)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Costo USD</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Lambda - requests</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>invocaciones x precio/request</t>
         </is>
       </c>
-      <c r="C4" s="11">
-        <f>Supuestos!$B$22*Supuestos!$B$5</f>
+      <c r="C4" s="6">
+        <f>Supuestos!$B$25*Supuestos!$B$5</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Lambda - computo (GB-s)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>inv x duracion(s) x memoria(GB) x precio/GB-s</t>
         </is>
       </c>
-      <c r="C5" s="11">
-        <f>Supuestos!$B$22*Supuestos!$B$23*Supuestos!$B$24*Supuestos!$B$6</f>
+      <c r="C5" s="6">
+        <f>Supuestos!$B$25*Supuestos!$B$26*Supuestos!$B$27*Supuestos!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Step Functions</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>transiciones x precio/transicion</t>
         </is>
       </c>
-      <c r="C6" s="11">
-        <f>Supuestos!$B$25*Supuestos!$B$7</f>
+      <c r="C6" s="6">
+        <f>Supuestos!$B$28*Supuestos!$B$7</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>API Gateway</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>requests x precio/request</t>
         </is>
       </c>
-      <c r="C7" s="11">
-        <f>Supuestos!$B$26*Supuestos!$B$8</f>
+      <c r="C7" s="6">
+        <f>Supuestos!$B$29*Supuestos!$B$8</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>DynamoDB - escrituras</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>escrituras x precio/WRU</t>
         </is>
       </c>
-      <c r="C8" s="11">
-        <f>Supuestos!$B$27*Supuestos!$B$9</f>
+      <c r="C8" s="6">
+        <f>Supuestos!$B$30*Supuestos!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>DynamoDB - lecturas</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>lecturas x precio/RRU</t>
         </is>
       </c>
-      <c r="C9" s="11">
-        <f>Supuestos!$B$28*Supuestos!$B$10</f>
+      <c r="C9" s="6">
+        <f>Supuestos!$B$31*Supuestos!$B$10</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>CloudWatch - logs</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>GB logs x precio/GB</t>
         </is>
       </c>
-      <c r="C10" s="11">
-        <f>Supuestos!$B$29*Supuestos!$B$12</f>
+      <c r="C10" s="6">
+        <f>Supuestos!$B$32*Supuestos!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Bedrock (segun modelo elegido)</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>IF Sonnet vs Haiku: tokens_in x precio_in + tokens_out x precio_out</t>
         </is>
       </c>
-      <c r="C11" s="11">
-        <f>IF(Supuestos!$B$36=1,Supuestos!$B$30*Supuestos!$B$15+Supuestos!$B$31*Supuestos!$B$16,Supuestos!$B$30*Supuestos!$B$17+Supuestos!$B$31*Supuestos!$B$18)</f>
+      <c r="C11" s="6">
+        <f>IF(Supuestos!$B$38=1,Supuestos!$B$33*Supuestos!$B$15+Supuestos!$B$34*Supuestos!$B$16,Supuestos!$B$33*Supuestos!$B$17+Supuestos!$B$34*Supuestos!$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WAF - requests (parte variable)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>(requests analisis / 1e6) x precio/millon  [despreciable por analisis]</t>
+        </is>
+      </c>
+      <c r="C12" s="6">
+        <f>(Supuestos!$B$29/1000000)*Supuestos!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>TOTAL variable por analisis</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>suma de los componentes de arriba</t>
         </is>
       </c>
-      <c r="C12" s="14">
-        <f>SUM(C4:C11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="C13" s="7">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Cambia el modelo en Supuestos (1=Sonnet, 2=Haiku) y veras recalcular Bedrock y el total.</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Cambia el modelo en Supuestos (1=Sonnet, 2=Haiku) y veras recalcular Bedrock y el total. WAF y Cognito son costos mayormente FIJOS/mes (ver hoja Costo mensual), no por analisis.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B14:C14"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1404,15 +1456,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Costo mensual estimado (variable + fijo)</t>
@@ -1420,122 +1472,167 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Formula</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>USD/mes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Variable: analisis del mes</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>analisis/mes x costo por analisis</t>
         </is>
       </c>
-      <c r="C4" s="16">
-        <f>Supuestos!$B$35*'Costo por analisis'!$C$12</f>
+      <c r="C4" s="8">
+        <f>Supuestos!$B$37*'Costo por analisis'!$C$13</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Fijo: Secrets Manager</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>secretos x precio/secreto-mes</t>
         </is>
       </c>
-      <c r="C5" s="16">
-        <f>Supuestos!$B$37*Supuestos!$B$14</f>
+      <c r="C5" s="8">
+        <f>Supuestos!$B$39*Supuestos!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Fijo: KMS</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>claves x precio/clave-mes</t>
         </is>
       </c>
-      <c r="C6" s="16">
-        <f>Supuestos!$B$38*Supuestos!$B$13</f>
+      <c r="C6" s="8">
+        <f>Supuestos!$B$40*Supuestos!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Fijo: Hosting CloudFront+S3</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>valor fijo editable en Supuestos</t>
         </is>
       </c>
-      <c r="C7" s="16">
-        <f>Supuestos!$B$39</f>
+      <c r="C7" s="8">
+        <f>Supuestos!$B$41</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fijo: WAF (web ACL + reglas)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>webACLs x precio_acl + reglas x precio_regla</t>
+        </is>
+      </c>
+      <c r="C8" s="8">
+        <f>Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Variable: WAF requests</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>millones_req x precio/millon</t>
+        </is>
+      </c>
+      <c r="C9" s="8">
+        <f>Supuestos!$B$44*Supuestos!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Variable: Cognito MAU</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MAU facturables x precio/MAU</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <f>Supuestos!$B$45*Supuestos!$B$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>TOTAL mensual estimado</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>suma variable + fijos</t>
         </is>
       </c>
-      <c r="C8" s="14">
-        <f>SUM(C4:C7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="C11" s="9">
+        <f>SUM(C4:C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Costo medio por analisis (incl. fijos)</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>total mensual / analisis del mes</t>
         </is>
       </c>
-      <c r="C10" s="14">
-        <f>C8/Supuestos!$B$35</f>
+      <c r="C13" s="10">
+        <f>C11/Supuestos!$B$37</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1549,10 +1646,10 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1563,87 +1660,83 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Sonnet (USD)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Haiku (USD)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Formula</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Tokens entrada</t>
         </is>
       </c>
-      <c r="B4" s="17">
-        <f>Supuestos!$B$30*Supuestos!$B$15</f>
-        <v/>
-      </c>
-      <c r="C4" s="17">
-        <f>Supuestos!$B$30*Supuestos!$B$17</f>
-        <v/>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="B4" s="6">
+        <f>Supuestos!$B$33*Supuestos!$B$15</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
+        <f>Supuestos!$B$33*Supuestos!$B$17</f>
+        <v/>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>tokens_in x precio_in</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Tokens salida</t>
         </is>
       </c>
-      <c r="B5" s="17">
-        <f>Supuestos!$B$31*Supuestos!$B$16</f>
-        <v/>
-      </c>
-      <c r="C5" s="17">
-        <f>Supuestos!$B$31*Supuestos!$B$18</f>
-        <v/>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="B5" s="6">
+        <f>Supuestos!$B$34*Supuestos!$B$16</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>Supuestos!$B$34*Supuestos!$B$18</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>tokens_out x precio_out</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Total Bedrock / analisis</t>
         </is>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="10">
         <f>SUM(B4:B5)</f>
         <v/>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="10">
         <f>SUM(C4:C5)</f>
         <v/>
       </c>
-      <c r="D6" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1658,14 +1751,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sensibilidad: costo mensual segun volumen de analisis</t>
@@ -1673,196 +1766,190 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Volumen base (editable):</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>&lt;- cambia este 50 y toda la tabla se recalcula</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Analisis/mes</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Variable (USD/mes)</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Fijos (USD/mes)</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Total (USD/mes)</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Costo medio/analisis</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="n">
+      <c r="A6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6">
         <f>$C$3*A6</f>
         <v/>
       </c>
-      <c r="C6" s="16">
-        <f>B6*'Costo por analisis'!$C$12</f>
-        <v/>
-      </c>
-      <c r="D6" s="16">
-        <f>(Supuestos!$B$37*Supuestos!$B$14+Supuestos!$B$38*Supuestos!$B$13+Supuestos!$B$39)</f>
-        <v/>
-      </c>
-      <c r="E6" s="14">
+      <c r="C6" s="8">
+        <f>B6*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>(Supuestos!$B$39*Supuestos!$B$14+Supuestos!$B$40*Supuestos!$B$13+Supuestos!$B$41+Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20+Supuestos!$B$44*Supuestos!$B$21+Supuestos!$B$45*Supuestos!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="23">
+      <c r="F6" s="10">
         <f>IF(B6=0,0,E6/B6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="n">
+      <c r="A7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7">
         <f>$C$3*A7</f>
         <v/>
       </c>
-      <c r="C7" s="16">
-        <f>B7*'Costo por analisis'!$C$12</f>
-        <v/>
-      </c>
-      <c r="D7" s="16">
-        <f>(Supuestos!$B$37*Supuestos!$B$14+Supuestos!$B$38*Supuestos!$B$13+Supuestos!$B$39)</f>
-        <v/>
-      </c>
-      <c r="E7" s="14">
+      <c r="C7" s="8">
+        <f>B7*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>(Supuestos!$B$39*Supuestos!$B$14+Supuestos!$B$40*Supuestos!$B$13+Supuestos!$B$41+Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20+Supuestos!$B$44*Supuestos!$B$21+Supuestos!$B$45*Supuestos!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E7" s="8">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="10">
         <f>IF(B7=0,0,E7/B7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8">
         <f>$C$3*A8</f>
         <v/>
       </c>
-      <c r="C8" s="16">
-        <f>B8*'Costo por analisis'!$C$12</f>
-        <v/>
-      </c>
-      <c r="D8" s="16">
-        <f>(Supuestos!$B$37*Supuestos!$B$14+Supuestos!$B$38*Supuestos!$B$13+Supuestos!$B$39)</f>
-        <v/>
-      </c>
-      <c r="E8" s="14">
+      <c r="C8" s="8">
+        <f>B8*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>(Supuestos!$B$39*Supuestos!$B$14+Supuestos!$B$40*Supuestos!$B$13+Supuestos!$B$41+Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20+Supuestos!$B$44*Supuestos!$B$21+Supuestos!$B$45*Supuestos!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="10">
         <f>IF(B8=0,0,E8/B8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n">
+      <c r="A9" t="n">
         <v>10</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9">
         <f>$C$3*A9</f>
         <v/>
       </c>
-      <c r="C9" s="16">
-        <f>B9*'Costo por analisis'!$C$12</f>
-        <v/>
-      </c>
-      <c r="D9" s="16">
-        <f>(Supuestos!$B$37*Supuestos!$B$14+Supuestos!$B$38*Supuestos!$B$13+Supuestos!$B$39)</f>
-        <v/>
-      </c>
-      <c r="E9" s="14">
+      <c r="C9" s="8">
+        <f>B9*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D9" s="8">
+        <f>(Supuestos!$B$39*Supuestos!$B$14+Supuestos!$B$40*Supuestos!$B$13+Supuestos!$B$41+Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20+Supuestos!$B$44*Supuestos!$B$21+Supuestos!$B$45*Supuestos!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E9" s="8">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="10">
         <f>IF(B9=0,0,E9/B9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n">
+      <c r="A10" t="n">
         <v>20</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10">
         <f>$C$3*A10</f>
         <v/>
       </c>
-      <c r="C10" s="16">
-        <f>B10*'Costo por analisis'!$C$12</f>
-        <v/>
-      </c>
-      <c r="D10" s="16">
-        <f>(Supuestos!$B$37*Supuestos!$B$14+Supuestos!$B$38*Supuestos!$B$13+Supuestos!$B$39)</f>
-        <v/>
-      </c>
-      <c r="E10" s="14">
+      <c r="C10" s="8">
+        <f>B10*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D10" s="8">
+        <f>(Supuestos!$B$39*Supuestos!$B$14+Supuestos!$B$40*Supuestos!$B$13+Supuestos!$B$41+Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20+Supuestos!$B$44*Supuestos!$B$21+Supuestos!$B$45*Supuestos!$B$22)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="10">
         <f>IF(B10=0,0,E10/B10)</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>La columna Factor multiplica el volumen base. Con base=50 veras 50, 100, 200, 500, 1000. El costo por analisis sale de la hoja 'Costo por analisis' (depende del modelo Bedrock elegido en Supuestos).</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>La columna Factor multiplica el volumen base. Con base=50 veras 50, 100, 200, 500, 1000. El costo por analisis sale de 'Costo por analisis'. Los Fijos ahora incluyen WAF y Cognito del To-Be.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="B12:F12"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1873,325 +1960,1436 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Verificacion vs AWS Pricing Calculator (200 analisis/mes, modelo Sonnet, us-east-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>URL de la estimacion en la calculadora de AWS (precios al 2026-10-16):</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://calculator.aws/#/estimate?id=9522a31ec4a7ecf35ed6def968263ccf9fd3711f</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Version con precios computados (Update+Share):</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://calculator.aws/#/estimate?id=0ea593458fbb3a44f0a11b361ff5b7e7261c5671</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Estimacion To-Be (incluye WAF + Cognito + Bedrock Sonnet, 200 analisis/mes, us-east-1):</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://calculator.aws/#/estimate?id=a2ab4d09438706b2e4a1ebaf9c3cf5d1a462ab8a</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Servicio</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Excel (USD/mes)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Calculadora (USD/mes)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Dif.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="8">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Calc muestra 0 (redondeo de su vista); real ~1.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Step Functions</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D10" s="8">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Calc aplica matiz de tier en transiciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>API Gateway</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ambos ~0 a este volumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CloudWatch</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="D12" s="8">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Calc suma cargo fijo de almacenamiento de logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DynamoDB</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Centavos; servicio sin campos expuestos en calc</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bedrock (Sonnet)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="C14" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="D14" s="8">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>COINCIDE (dif. por redondeo de tokens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Secrets Manager</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="D15" s="8">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Calc suma llamadas API</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KMS</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="D16" s="8">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Calc suma requests simetricas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WAF (To-Be)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>por verificar</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>web ACL 5 + 3 reglas 3 + 0.5M req 0.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cognito (To-Be)</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>por verificar</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>MAU dentro de capa gratis Essentials en escenario base</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hosting CloudFront+S3</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Fijo estimado</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B20" s="12">
+        <f>SUM(B9:B19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Conclusion:</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>El To-Be agrega WAF (~US$8/mes fijo) y Cognito (~0 en volumen bajo, crece con MAU). Los componentes dominantes del As-Is (Bedrock, CloudWatch, Secrets, KMS) ya estaban verificados contra la calculadora con diferencias de centavos. Pendiente: nueva estimacion en la calculadora incluyendo WAF+Cognito.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verificacion vs AWS Pricing Calculator (200 analisis/mes, modelo Sonnet, us-east-1)</t>
+          <t>Costos AWS por ambiente (Produccion vs Staging)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>URL de la estimacion en la calculadora de AWS (precios al 2026-10-16):</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="25" t="inlineStr">
-        <is>
-          <t>https://calculator.aws/#/estimate?id=9522a31ec4a7ecf35ed6def968263ccf9fd3711f</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Produccion = 200 analisis/mes (celda Supuestos B37). Staging = volumen editable abajo.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Version con precios computados (Update+Share):</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PARAMETROS STAGING (editables)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>https://calculator.aws/#/estimate?id=0ea593458fbb3a44f0a11b361ff5b7e7261c5671</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Analisis por mes (staging)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WAF: web ACLs (staging)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>Servicio</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Excel (USD/mes)</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Calculadora (USD/mes)</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Dif.</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WAF: reglas/grupos (staging)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Lambda</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="28">
-        <f>C8-B8</f>
-        <v/>
-      </c>
-      <c r="E8" s="29" t="inlineStr">
-        <is>
-          <t>Calc muestra 0 (redondeo de su vista); el valor real ~1.40 esta en el Excel</t>
-        </is>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WAF: requests/mes millones (staging)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Step Functions</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C9" s="27" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D9" s="30">
-        <f>C9-B9</f>
-        <v/>
-      </c>
-      <c r="E9" s="29" t="inlineStr">
-        <is>
-          <t>Calc aplica matiz de tier en transiciones</t>
-        </is>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hosting CloudFront+S3 (staging)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>API Gateway</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="30">
-        <f>C10-B10</f>
-        <v/>
-      </c>
-      <c r="E10" s="29" t="inlineStr">
-        <is>
-          <t>Ambos ~0 a este volumen</t>
-        </is>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Secretos almacenados (staging)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>CloudWatch</t>
-        </is>
-      </c>
-      <c r="B11" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="27" t="n">
-        <v>5.05</v>
-      </c>
-      <c r="D11" s="30">
-        <f>C11-B11</f>
-        <v/>
-      </c>
-      <c r="E11" s="29" t="inlineStr">
-        <is>
-          <t>Calc suma cargo fijo de almacenamiento de logs</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>DynamoDB</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="D12" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" s="29" t="inlineStr">
-        <is>
-          <t>No modelado en calc (servicio sin campos expuestos); centavos</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Claves KMS (staging)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Bedrock (Sonnet)</t>
-        </is>
-      </c>
-      <c r="B13" s="27" t="n">
-        <v>21</v>
-      </c>
-      <c r="C13" s="27" t="n">
-        <v>20.99</v>
-      </c>
-      <c r="D13" s="30">
-        <f>C13-B13</f>
-        <v/>
-      </c>
-      <c r="E13" s="29" t="inlineStr">
-        <is>
-          <t>COINCIDE (dif. por redondeo de tokens)</t>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Produccion (USD/mes)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Staging (USD/mes)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Formula base</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Secrets Manager</t>
-        </is>
-      </c>
-      <c r="B14" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="C14" s="27" t="n">
-        <v>4.05</v>
-      </c>
-      <c r="D14" s="30">
-        <f>C14-B14</f>
-        <v/>
-      </c>
-      <c r="E14" s="29" t="inlineStr">
-        <is>
-          <t>Calc suma llamadas API</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Variable: analisis del mes</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>Supuestos!$B$37*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="C14" s="8">
+        <f>$B$5*'Costo por analisis'!$C$13</f>
+        <v/>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>analisis x costo/analisis</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>KMS</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="27" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="D15" s="30">
-        <f>C15-B15</f>
-        <v/>
-      </c>
-      <c r="E15" s="29" t="inlineStr">
-        <is>
-          <t>Calc suma requests simetricas</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fijo: Secrets Manager</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>Supuestos!$B$39*Supuestos!$B$14</f>
+        <v/>
+      </c>
+      <c r="C15" s="8">
+        <f>$B$10*Supuestos!$B$14</f>
+        <v/>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>secretos x precio</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Hosting CloudFront+S3</t>
-        </is>
-      </c>
-      <c r="B16" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E16" s="29" t="inlineStr">
-        <is>
-          <t>Fijo estimado; no incluido en esta estimacion de calc</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fijo: KMS</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>Supuestos!$B$40*Supuestos!$B$13</f>
+        <v/>
+      </c>
+      <c r="C16" s="8">
+        <f>$B$11*Supuestos!$B$13</f>
+        <v/>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>claves x precio</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Fijo: Hosting CloudFront+S3</t>
+        </is>
+      </c>
+      <c r="B17" s="8">
+        <f>Supuestos!$B$41</f>
+        <v/>
+      </c>
+      <c r="C17" s="8">
+        <f>$B$9</f>
+        <v/>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>valor fijo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fijo: WAF (web ACL + reglas)</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20</f>
+        <v/>
+      </c>
+      <c r="C18" s="8">
+        <f>$B$6*Supuestos!$B$19+$B$7*Supuestos!$B$20</f>
+        <v/>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ACLs x precio + reglas x precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Variable: WAF requests</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>Supuestos!$B$44*Supuestos!$B$21</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>$B$8*Supuestos!$B$21</f>
+        <v/>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>millones req x precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Variable: Cognito MAU</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>Supuestos!$B$45*Supuestos!$B$22</f>
+        <v/>
+      </c>
+      <c r="C20" s="8">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MAU x precio (staging ~0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL AWS por ambiente</t>
+        </is>
+      </c>
+      <c r="B21" s="13">
+        <f>SUM(B14:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="13">
+        <f>SUM(C14:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CONSOLIDADO AWS (Prod + Staging)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Total AWS mensual (ambos ambientes)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>B21+C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Total AWS anual (ambos ambientes)</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>B24*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Equivalente COP/mes (TRM 3500)</t>
+        </is>
+      </c>
+      <c r="B26" s="14">
+        <f>B24*3500</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Inversion inicial y gastos operativos (OPEX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>INVERSION INICIAL (una vez)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Horas de desarrollo</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Horas otras areas</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tarifa (USD/hora)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Horas totales</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>B4+B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Costo total desarrollo (USD)</t>
+        </is>
+      </c>
+      <c r="C8" s="15">
+        <f>(B4+B5)*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Equivalente COP (TRM 3500)</t>
+        </is>
+      </c>
+      <c r="C9" s="14">
+        <f>C8*3500</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>OPEX RECURRENTE</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>USD/mes</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>USD/anio</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AWS (Prod + Staging)</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>Ambientes!$B$24</f>
+        <v/>
+      </c>
+      <c r="C12" s="8">
+        <f>B12*12</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>consolidado hoja Ambientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Kiro (plan Power)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C13" s="8">
+        <f>B13*12</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>USD$200/mes, 10k creditos (uso ~1.500/mes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OPEX TOTAL</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>B12+B13</f>
+        <v/>
+      </c>
+      <c r="C14" s="9">
+        <f>C12+C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OPEX TOTAL COP/mes (TRM 3500)</t>
+        </is>
+      </c>
+      <c r="B15" s="14">
+        <f>B14*3500</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Kiro Power incluye 10.000 creditos; el uso previsto (~1.500/mes) cabe en planes menores. Se usa Power por indicacion del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B17:D18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Resumen financiero (3 escenarios, horizonte 3 anios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Moneda USD | TRM COP 3500 | Tasa de descuento (editable):</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SUPUESTOS DE INGRESO (editables)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Optimista</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ARPU (USD/cuenta/mes)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cuentas activas Ano 1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cuentas activas Ano 2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cuentas activas Ano 3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ingresos Ano 1 (USD)</t>
+        </is>
+      </c>
+      <c r="B10" s="14">
+        <f>B6*B5*12</f>
+        <v/>
+      </c>
+      <c r="C10" s="14">
+        <f>C6*C5*12</f>
+        <v/>
+      </c>
+      <c r="D10" s="14">
+        <f>D6*D5*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ingresos Ano 2 (USD)</t>
+        </is>
+      </c>
+      <c r="B11" s="14">
+        <f>B7*B5*12</f>
+        <v/>
+      </c>
+      <c r="C11" s="14">
+        <f>C7*C5*12</f>
+        <v/>
+      </c>
+      <c r="D11" s="14">
+        <f>D7*D5*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ingresos Ano 3 (USD)</t>
+        </is>
+      </c>
+      <c r="B12" s="14">
+        <f>B8*B5*12</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>C8*C5*12</f>
+        <v/>
+      </c>
+      <c r="D12" s="14">
+        <f>D8*D5*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OPEX Ano 1 (USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="14">
+        <f>'Inversion y OPEX'!$C$14</f>
+        <v/>
+      </c>
+      <c r="C13" s="14">
+        <f>'Inversion y OPEX'!$C$14</f>
+        <v/>
+      </c>
+      <c r="D13" s="14">
+        <f>'Inversion y OPEX'!$C$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OPEX Ano 2 (USD)</t>
+        </is>
+      </c>
+      <c r="B14" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.12</f>
+        <v/>
+      </c>
+      <c r="C14" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.12</f>
+        <v/>
+      </c>
+      <c r="D14" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OPEX Ano 3 (USD)</t>
+        </is>
+      </c>
+      <c r="B15" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.25</f>
+        <v/>
+      </c>
+      <c r="C15" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.25</f>
+        <v/>
+      </c>
+      <c r="D15" s="14">
+        <f>'Inversion y OPEX'!$C$14*1.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EBITDA Ano 1 (USD)</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>B10-B13</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>C10-C13</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>D10-D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EBITDA Ano 2 (USD)</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>SUM(B8:B16)</f>
+        <f>B11-B14</f>
         <v/>
       </c>
       <c r="C17" s="14">
-        <f>C8+C9+C10+C11+C13+C14+C15</f>
-        <v/>
-      </c>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>Total calc = 31.25 (sin DynamoDB ni Hosting). Excel incluye esos dos.</t>
-        </is>
+        <f>C11-C14</f>
+        <v/>
+      </c>
+      <c r="D17" s="14">
+        <f>D11-D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EBITDA Ano 3 (USD)</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>B12-B15</f>
+        <v/>
+      </c>
+      <c r="C18" s="14">
+        <f>C12-C15</f>
+        <v/>
+      </c>
+      <c r="D18" s="14">
+        <f>D12-D15</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Conclusion:</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>Los componentes dominantes (Bedrock ~21, CloudWatch ~5, Secrets ~4, KMS ~1) coinciden con la calculadora de AWS con diferencias de centavos. Las diferencias restantes se explican por: (1) la calculadora muestra Lambda en 0 por redondeo de su vista; (2) hosting CloudFront+S3 y DynamoDB no se incluyeron en esa estimacion. Excel y calculadora son consistentes para decisiones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Inversion inicial (USD)</t>
+        </is>
+      </c>
+      <c r="B19" s="14">
+        <f>'Inversion y OPEX'!$C$8</f>
+        <v/>
+      </c>
+      <c r="C19" s="14">
+        <f>'Inversion y OPEX'!$C$8</f>
+        <v/>
+      </c>
+      <c r="D19" s="14">
+        <f>'Inversion y OPEX'!$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>INDICADORES</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Conservador</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Optimista</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EBITDA acumulado 3 anios</t>
+        </is>
+      </c>
+      <c r="B22" s="14">
+        <f>SUM(B16:B18)</f>
+        <v/>
+      </c>
+      <c r="C22" s="14">
+        <f>SUM(C16:C18)</f>
+        <v/>
+      </c>
+      <c r="D22" s="14">
+        <f>SUM(D16:D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ROI 3 anios (%)</t>
+        </is>
+      </c>
+      <c r="B23" s="17">
+        <f>(B22-B19)/B19</f>
+        <v/>
+      </c>
+      <c r="C23" s="17">
+        <f>(C22-C19)/C19</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>(D22-D19)/D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>VPN (USD)</t>
+        </is>
+      </c>
+      <c r="B24" s="14">
+        <f>-B19 + B16/(1+$E$2) + B17/(1+$E$2)^2 + B18/(1+$E$2)^3</f>
+        <v/>
+      </c>
+      <c r="C24" s="14">
+        <f>-C19 + C16/(1+$E$2) + C17/(1+$E$2)^2 + C18/(1+$E$2)^3</f>
+        <v/>
+      </c>
+      <c r="D24" s="14">
+        <f>-D19 + D16/(1+$E$2) + D17/(1+$E$2)^2 + D18/(1+$E$2)^3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TIR (%)</t>
+        </is>
+      </c>
+      <c r="B25" s="17">
+        <f>IRR(B28:B31)</f>
+        <v/>
+      </c>
+      <c r="C25" s="17">
+        <f>IRR(C28:C31)</f>
+        <v/>
+      </c>
+      <c r="D25" s="17">
+        <f>IRR(D28:D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Payback simple (meses, base EBITDA Ano 1)</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>B19/(B16/12)</f>
+        <v/>
+      </c>
+      <c r="C26" s="18">
+        <f>C19/(C16/12)</f>
+        <v/>
+      </c>
+      <c r="D26" s="18">
+        <f>D19/(D16/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Flujo 0 (=-inversion)</t>
+        </is>
+      </c>
+      <c r="B28" s="14">
+        <f>-B19</f>
+        <v/>
+      </c>
+      <c r="C28" s="14">
+        <f>-C19</f>
+        <v/>
+      </c>
+      <c r="D28" s="14">
+        <f>-D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Flujo Ano 1</t>
+        </is>
+      </c>
+      <c r="B29" s="14">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="C29" s="14">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="D29" s="14">
+        <f>D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Flujo Ano 2</t>
+        </is>
+      </c>
+      <c r="B30" s="14">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C30" s="14">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="D30" s="14">
+        <f>D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Flujo Ano 3</t>
+        </is>
+      </c>
+      <c r="B31" s="14">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="C31" s="14">
+        <f>C18</f>
+        <v/>
+      </c>
+      <c r="D31" s="14">
+        <f>D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Nota: ROI = (EBITDA acumulado - inversion)/inversion. VPN descuenta los EBITDA anuales a la tasa editable (E2). TIR via IRR sobre flujos anuales (filas 28-31). El Payback simple usa el EBITDA mensual del Ano 1 (metodo conservador/lineal); el payback real considerando el crecimiento de los Anos 2-3 es menor (ver documento de analisis). Cambia ARPU, cuentas o la tasa y todo recalcula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="B19:E21"/>
-    <mergeCell ref="A3:E3"/>
+  <mergeCells count="1">
+    <mergeCell ref="A33:E35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(costos): alinear WAF a 1M requests y actualizar URL de la calculadora AWS
</commit_message>
<xml_diff>
--- a/docs/gfourmis-sesion-arquitectura/AutoWAR-Estimacion-Costos.xlsx
+++ b/docs/gfourmis-sesion-arquitectura/AutoWAR-Estimacion-Costos.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="3816" windowWidth="23256" windowHeight="12696" tabRatio="600" firstSheet="1" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costo por analisis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costo mensual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa Bedrock" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa Bedrock" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costo mensual" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidad" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verif. Calculadora AWS" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ambientes" sheetId="7" state="visible" r:id="rId7"/>
@@ -18,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Financiero" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -39,15 +38,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00B85450"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -59,22 +65,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEEE"/>
+        <fgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
+        <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,23 +94,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -118,7 +126,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,9 +133,15 @@
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -492,23 +505,23 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="2"/>
+    <col width="18" customWidth="1" style="19" min="3" max="3"/>
+    <col width="46" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>AutoWAR - Supuestos de costo (celdas AMARILLAS = editables)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="75" customHeight="1" s="19">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Region: us-east-1 | Moneda: USD | Precios de referencia publicos (oct-2026). Incluye componentes To-Be (WAF, Cognito, Lambda Authorizer, entitlements). Validar en la calculadora AWS para cotizacion formal.</t>
         </is>
@@ -550,7 +563,7 @@
           <t>USD/request</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>US$0.20 por 1M requests</t>
         </is>
@@ -570,7 +583,7 @@
           <t>USD/GB-s</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>x86 on-demand</t>
         </is>
@@ -590,7 +603,7 @@
           <t>USD/transicion</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>US$0.025 por 1.000 transiciones</t>
         </is>
@@ -610,7 +623,7 @@
           <t>USD/request</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>US$3.50 por 1M requests</t>
         </is>
@@ -630,7 +643,7 @@
           <t>USD/escritura</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>US$1.25 por 1M WRU</t>
         </is>
@@ -650,7 +663,7 @@
           <t>USD/lectura</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>US$0.25 por 1M RRU</t>
         </is>
@@ -670,7 +683,7 @@
           <t>USD/GB-mes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>S3 Standard</t>
         </is>
@@ -690,7 +703,7 @@
           <t>USD/GB</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>ingestion de logs</t>
         </is>
@@ -710,7 +723,7 @@
           <t>USD/clave-mes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>clave gestionada</t>
         </is>
@@ -730,7 +743,7 @@
           <t>USD/secreto-mes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>+US$0.05 por 10k llamadas (despreciable)</t>
         </is>
@@ -750,7 +763,7 @@
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>US$3 por 1M tokens in</t>
         </is>
@@ -770,7 +783,7 @@
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>US$15 por 1M tokens out</t>
         </is>
@@ -790,7 +803,7 @@
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>~US$0.80 por 1M tokens in</t>
         </is>
@@ -810,7 +823,7 @@
           <t>USD/token</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>~US$4 por 1M tokens out</t>
         </is>
@@ -830,7 +843,7 @@
           <t>USD/web ACL-mes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>US$5 por web ACL/mes</t>
         </is>
@@ -850,7 +863,7 @@
           <t>USD/regla-mes</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>US$1 por regla o managed rule group/mes</t>
         </is>
@@ -870,13 +883,13 @@
           <t>USD/millon req</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>US$0.60 por 1M requests inspeccionados</t>
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="30" customHeight="1" s="19">
       <c r="A22" t="inlineStr">
         <is>
           <t>Cognito: por MAU (sobre capa gratis)</t>
@@ -890,7 +903,7 @@
           <t>USD/MAU</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Essentials ~US$0.015/MAU; 10k MAU gratis (fed. menor)</t>
         </is>
@@ -932,7 +945,7 @@
           <t>invocaciones</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>6 pilares + orquestador + authorizer</t>
         </is>
@@ -952,7 +965,7 @@
           <t>segundos</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>editable segun cuenta</t>
         </is>
@@ -972,7 +985,7 @@
           <t>GB</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>1024 MB</t>
         </is>
@@ -992,7 +1005,7 @@
           <t>transiciones</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>fan-out + joins</t>
         </is>
@@ -1012,7 +1025,7 @@
           <t>requests</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>validar + analizar + polling</t>
         </is>
@@ -1032,7 +1045,7 @@
           <t>escrituras</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>resultados + items por pilar + entitlements</t>
         </is>
@@ -1052,7 +1065,7 @@
           <t>lecturas</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>resultados + lectura de entitlements</t>
         </is>
@@ -1072,7 +1085,7 @@
           <t>GB</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="18" t="inlineStr">
         <is>
           <t>~50 MB de logs por analisis</t>
         </is>
@@ -1092,7 +1105,7 @@
           <t>tokens</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>hallazgos + contexto</t>
         </is>
@@ -1112,7 +1125,7 @@
           <t>tokens</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>resumen redactado</t>
         </is>
@@ -1207,7 +1220,7 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -1242,14 +1255,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" style="19" min="1" max="1"/>
+    <col width="52" customWidth="1" style="19" min="2" max="2"/>
+    <col width="14" customWidth="1" style="19" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Costo variable por 1 analisis (1 cuenta, 6 pilares)</t>
@@ -1279,7 +1292,7 @@
           <t>Lambda - requests</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>invocaciones x precio/request</t>
         </is>
@@ -1295,7 +1308,7 @@
           <t>Lambda - computo (GB-s)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>inv x duracion(s) x memoria(GB) x precio/GB-s</t>
         </is>
@@ -1311,7 +1324,7 @@
           <t>Step Functions</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>transiciones x precio/transicion</t>
         </is>
@@ -1327,7 +1340,7 @@
           <t>API Gateway</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>requests x precio/request</t>
         </is>
@@ -1343,7 +1356,7 @@
           <t>DynamoDB - escrituras</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>escrituras x precio/WRU</t>
         </is>
@@ -1359,7 +1372,7 @@
           <t>DynamoDB - lecturas</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>lecturas x precio/RRU</t>
         </is>
@@ -1375,7 +1388,7 @@
           <t>CloudWatch - logs</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>GB logs x precio/GB</t>
         </is>
@@ -1385,13 +1398,13 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="30" customHeight="1" s="19">
       <c r="A11" t="inlineStr">
         <is>
           <t>Bedrock (segun modelo elegido)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>IF Sonnet vs Haiku: tokens_in x precio_in + tokens_out x precio_out</t>
         </is>
@@ -1401,13 +1414,13 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="30" customHeight="1" s="19">
       <c r="A12" t="inlineStr">
         <is>
           <t>WAF - requests (parte variable)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>(requests analisis / 1e6) x precio/millon  [despreciable por analisis]</t>
         </is>
@@ -1433,13 +1446,13 @@
         <v/>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="60" customHeight="1" s="19">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Cambia el modelo en Supuestos (1=Sonnet, 2=Haiku) y veras recalcular Bedrock y el total. WAF y Cognito son costos mayormente FIJOS/mes (ver hoja Costo mensual), no por analisis.</t>
         </is>
@@ -1456,18 +1469,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="3"/>
+    <col width="26" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Costo mensual estimado (variable + fijo)</t>
+          <t>Bedrock por analisis: Sonnet vs Haiku</t>
         </is>
       </c>
     </row>
@@ -1479,156 +1492,72 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
+          <t>Sonnet (USD)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Haiku (USD)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>Formula</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>USD/mes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Variable: analisis del mes</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>analisis/mes x costo por analisis</t>
-        </is>
-      </c>
-      <c r="C4" s="8">
-        <f>Supuestos!$B$37*'Costo por analisis'!$C$13</f>
-        <v/>
+          <t>Tokens entrada</t>
+        </is>
+      </c>
+      <c r="B4" s="6">
+        <f>Supuestos!$B$33*Supuestos!$B$15</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
+        <f>Supuestos!$B$33*Supuestos!$B$17</f>
+        <v/>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>tokens_in x precio_in</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fijo: Secrets Manager</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>secretos x precio/secreto-mes</t>
-        </is>
-      </c>
-      <c r="C5" s="8">
-        <f>Supuestos!$B$39*Supuestos!$B$14</f>
-        <v/>
+          <t>Tokens salida</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>Supuestos!$B$34*Supuestos!$B$16</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>Supuestos!$B$34*Supuestos!$B$18</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>tokens_out x precio_out</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Fijo: KMS</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>claves x precio/clave-mes</t>
-        </is>
-      </c>
-      <c r="C6" s="8">
-        <f>Supuestos!$B$40*Supuestos!$B$13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Fijo: Hosting CloudFront+S3</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>valor fijo editable en Supuestos</t>
-        </is>
-      </c>
-      <c r="C7" s="8">
-        <f>Supuestos!$B$41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Fijo: WAF (web ACL + reglas)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>webACLs x precio_acl + reglas x precio_regla</t>
-        </is>
-      </c>
-      <c r="C8" s="8">
-        <f>Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Variable: WAF requests</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>millones_req x precio/millon</t>
-        </is>
-      </c>
-      <c r="C9" s="8">
-        <f>Supuestos!$B$44*Supuestos!$B$21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Variable: Cognito MAU</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MAU facturables x precio/MAU</t>
-        </is>
-      </c>
-      <c r="C10" s="8">
-        <f>Supuestos!$B$45*Supuestos!$B$22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL mensual estimado</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>suma variable + fijos</t>
-        </is>
-      </c>
-      <c r="C11" s="9">
-        <f>SUM(C4:C10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Costo medio por analisis (incl. fijos)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>total mensual / analisis del mes</t>
-        </is>
-      </c>
-      <c r="C13" s="10">
-        <f>C11/Supuestos!$B$37</f>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Total Bedrock / analisis</t>
+        </is>
+      </c>
+      <c r="B6" s="10">
+        <f>SUM(B4:B5)</f>
+        <v/>
+      </c>
+      <c r="C6" s="10">
+        <f>SUM(C4:C5)</f>
         <v/>
       </c>
     </row>
@@ -1643,19 +1572,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" style="19" min="1" max="1"/>
+    <col width="42" customWidth="1" style="19" min="2" max="2"/>
+    <col width="14" customWidth="1" style="19" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bedrock por analisis: Sonnet vs Haiku</t>
+          <t>Costo mensual estimado (variable + fijo)</t>
         </is>
       </c>
     </row>
@@ -1667,72 +1595,156 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Sonnet (USD)</t>
+          <t>Formula</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Haiku (USD)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Formula</t>
+          <t>USD/mes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tokens entrada</t>
-        </is>
-      </c>
-      <c r="B4" s="6">
-        <f>Supuestos!$B$33*Supuestos!$B$15</f>
-        <v/>
-      </c>
-      <c r="C4" s="6">
-        <f>Supuestos!$B$33*Supuestos!$B$17</f>
-        <v/>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>tokens_in x precio_in</t>
-        </is>
+          <t>Variable: analisis del mes</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>analisis/mes x costo por analisis</t>
+        </is>
+      </c>
+      <c r="C4" s="8">
+        <f>Supuestos!$B$37*'Costo por analisis'!$C$13</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tokens salida</t>
-        </is>
-      </c>
-      <c r="B5" s="6">
-        <f>Supuestos!$B$34*Supuestos!$B$16</f>
-        <v/>
-      </c>
-      <c r="C5" s="6">
-        <f>Supuestos!$B$34*Supuestos!$B$18</f>
-        <v/>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>tokens_out x precio_out</t>
-        </is>
+          <t>Fijo: Secrets Manager</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>secretos x precio/secreto-mes</t>
+        </is>
+      </c>
+      <c r="C5" s="8">
+        <f>Supuestos!$B$39*Supuestos!$B$14</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Total Bedrock / analisis</t>
-        </is>
-      </c>
-      <c r="B6" s="10">
-        <f>SUM(B4:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="10">
-        <f>SUM(C4:C5)</f>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fijo: KMS</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>claves x precio/clave-mes</t>
+        </is>
+      </c>
+      <c r="C6" s="8">
+        <f>Supuestos!$B$40*Supuestos!$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fijo: Hosting CloudFront+S3</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>valor fijo editable en Supuestos</t>
+        </is>
+      </c>
+      <c r="C7" s="8">
+        <f>Supuestos!$B$41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fijo: WAF (web ACL + reglas)</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>webACLs x precio_acl + reglas x precio_regla</t>
+        </is>
+      </c>
+      <c r="C8" s="8">
+        <f>Supuestos!$B$42*Supuestos!$B$19+Supuestos!$B$43*Supuestos!$B$20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Variable: WAF requests</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>millones_req x precio/millon</t>
+        </is>
+      </c>
+      <c r="C9" s="8">
+        <f>Supuestos!$B$44*Supuestos!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Variable: Cognito MAU</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>MAU facturables x precio/MAU</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <f>Supuestos!$B$45*Supuestos!$B$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL mensual estimado</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>suma variable + fijos</t>
+        </is>
+      </c>
+      <c r="C11" s="9">
+        <f>SUM(C4:C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Costo medio por analisis (incl. fijos)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>total mensual / analisis del mes</t>
+        </is>
+      </c>
+      <c r="C13" s="10">
+        <f>C11/Supuestos!$B$37</f>
         <v/>
       </c>
     </row>
@@ -1748,17 +1760,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="2"/>
+    <col width="18" customWidth="1" style="19" min="3" max="3"/>
+    <col width="16" customWidth="1" style="19" min="4" max="5"/>
+    <col width="20" customWidth="1" style="19" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sensibilidad: costo mensual segun volumen de analisis</t>
@@ -1937,13 +1948,13 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="210" customHeight="1" s="19">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>La columna Factor multiplica el volumen base. Con base=50 veras 50, 100, 200, 500, 1000. El costo por analisis sale de 'Costo por analisis'. Los Fijos ahora incluyen WAF y Cognito del To-Be.</t>
         </is>
@@ -1961,16 +1972,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="2"/>
+    <col width="20" customWidth="1" style="19" min="3" max="3"/>
+    <col width="10" customWidth="1" style="19" min="4" max="4"/>
+    <col width="52" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Verificacion vs AWS Pricing Calculator (200 analisis/mes, modelo Sonnet, us-east-1)</t>
@@ -2013,9 +2024,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>https://calculator.aws/#/estimate?id=a2ab4d09438706b2e4a1ebaf9c3cf5d1a462ab8a</t>
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>https://calculator.aws/#/estimate?id=8748b8884c260d78b625d6ce3fbf631f45f8e552</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2073,7 @@
         <f>C9-B9</f>
         <v/>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Calc muestra 0 (redondeo de su vista); real ~1.40</t>
         </is>
@@ -2084,7 +2095,7 @@
         <f>C10-B10</f>
         <v/>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Calc aplica matiz de tier en transiciones</t>
         </is>
@@ -2106,7 +2117,7 @@
         <f>C11-B11</f>
         <v/>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Ambos ~0 a este volumen</t>
         </is>
@@ -2128,7 +2139,7 @@
         <f>C12-B12</f>
         <v/>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>Calc suma cargo fijo de almacenamiento de logs</t>
         </is>
@@ -2153,7 +2164,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Centavos; servicio sin campos expuestos en calc</t>
         </is>
@@ -2175,7 +2186,7 @@
         <f>C14-B14</f>
         <v/>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>COINCIDE (dif. por redondeo de tokens)</t>
         </is>
@@ -2197,7 +2208,7 @@
         <f>C15-B15</f>
         <v/>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>Calc suma llamadas API</t>
         </is>
@@ -2219,7 +2230,7 @@
         <f>C16-B16</f>
         <v/>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>Calc suma requests simetricas</t>
         </is>
@@ -2244,9 +2255,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>web ACL 5 + 3 reglas 3 + 0.5M req 0.30</t>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>web ACL 5 + 3 reglas 3 + 1M req 0.60</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2280,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>MAU dentro de capa gratis Essentials en escenario base</t>
         </is>
@@ -2294,7 +2305,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>Fijo estimado</t>
         </is>
@@ -2306,24 +2317,27 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="11">
         <f>SUM(B9:B19)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="360" customHeight="1" s="19">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Conclusion:</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>El To-Be agrega WAF (~US$8/mes fijo) y Cognito (~0 en volumen bajo, crece con MAU). Los componentes dominantes del As-Is (Bedrock, CloudWatch, Secrets, KMS) ya estaban verificados contra la calculadora con diferencias de centavos. Pendiente: nueva estimacion en la calculadora incluyendo WAF+Cognito.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" location="/estimate?id=8748b8884c260d78b625d6ce3fbf631f45f8e552" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2335,23 +2349,22 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" style="19" min="1" max="1"/>
+    <col width="18" customWidth="1" style="19" min="2" max="3"/>
+    <col width="16" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Costos AWS por ambiente (Produccion vs Staging)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="45" customHeight="1" s="19">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Produccion = 200 analisis/mes (celda Supuestos B37). Staging = volumen editable abajo.</t>
         </is>
@@ -2607,11 +2620,11 @@
           <t>TOTAL AWS por ambiente</t>
         </is>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="12">
         <f>SUM(B14:B20)</f>
         <v/>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="12">
         <f>SUM(C14:C20)</f>
         <v/>
       </c>
@@ -2651,7 +2664,7 @@
           <t>Equivalente COP/mes (TRM 3500)</t>
         </is>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="13">
         <f>B24*3500</f>
         <v/>
       </c>
@@ -2668,15 +2681,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" style="19" min="1" max="1"/>
+    <col width="18" customWidth="1" style="19" min="2" max="3"/>
+    <col width="30" customWidth="1" style="19" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Inversion inicial y gastos operativos (OPEX)</t>
@@ -2752,7 +2764,7 @@
           <t>Costo total desarrollo (USD)</t>
         </is>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="14">
         <f>(B4+B5)*B6</f>
         <v/>
       </c>
@@ -2763,7 +2775,7 @@
           <t>Equivalente COP (TRM 3500)</t>
         </is>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="13">
         <f>C8*3500</f>
         <v/>
       </c>
@@ -2850,7 +2862,7 @@
           <t>OPEX TOTAL COP/mes (TRM 3500)</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="13">
         <f>B14*3500</f>
         <v/>
       </c>
@@ -2861,7 +2873,7 @@
           <t>Nota</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Kiro Power incluye 10.000 creditos; el uso previsto (~1.500/mes) cabe en planes menores. Se usa Power por indicacion del equipo.</t>
         </is>
@@ -2883,16 +2895,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="4"/>
+    <col width="28" customWidth="1" style="19" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17.25" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Resumen financiero (3 escenarios, horizonte 3 anios)</t>
@@ -2905,7 +2915,7 @@
           <t>Moneda USD | TRM COP 3500 | Tasa de descuento (editable):</t>
         </is>
       </c>
-      <c r="E2" s="16" t="n">
+      <c r="E2" s="15" t="n">
         <v>0.14</v>
       </c>
     </row>
@@ -3001,15 +3011,15 @@
           <t>Ingresos Ano 1 (USD)</t>
         </is>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="13">
         <f>B6*B5*12</f>
         <v/>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="13">
         <f>C6*C5*12</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="13">
         <f>D6*D5*12</f>
         <v/>
       </c>
@@ -3020,15 +3030,15 @@
           <t>Ingresos Ano 2 (USD)</t>
         </is>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="13">
         <f>B7*B5*12</f>
         <v/>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="13">
         <f>C7*C5*12</f>
         <v/>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="13">
         <f>D7*D5*12</f>
         <v/>
       </c>
@@ -3039,15 +3049,15 @@
           <t>Ingresos Ano 3 (USD)</t>
         </is>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="13">
         <f>B8*B5*12</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="13">
         <f>C8*C5*12</f>
         <v/>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="13">
         <f>D8*D5*12</f>
         <v/>
       </c>
@@ -3058,15 +3068,15 @@
           <t>OPEX Ano 1 (USD)</t>
         </is>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="13">
         <f>'Inversion y OPEX'!$C$14</f>
         <v/>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="13">
         <f>'Inversion y OPEX'!$C$14</f>
         <v/>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="13">
         <f>'Inversion y OPEX'!$C$14</f>
         <v/>
       </c>
@@ -3077,15 +3087,15 @@
           <t>OPEX Ano 2 (USD)</t>
         </is>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="13">
         <f>'Inversion y OPEX'!$C$14*1.12</f>
         <v/>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="13">
         <f>'Inversion y OPEX'!$C$14*1.12</f>
         <v/>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="13">
         <f>'Inversion y OPEX'!$C$14*1.12</f>
         <v/>
       </c>
@@ -3096,15 +3106,15 @@
           <t>OPEX Ano 3 (USD)</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="13">
         <f>'Inversion y OPEX'!$C$14*1.25</f>
         <v/>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="13">
         <f>'Inversion y OPEX'!$C$14*1.25</f>
         <v/>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="13">
         <f>'Inversion y OPEX'!$C$14*1.25</f>
         <v/>
       </c>
@@ -3115,15 +3125,15 @@
           <t>EBITDA Ano 1 (USD)</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="13">
         <f>B10-B13</f>
         <v/>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="13">
         <f>C10-C13</f>
         <v/>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="13">
         <f>D10-D13</f>
         <v/>
       </c>
@@ -3134,15 +3144,15 @@
           <t>EBITDA Ano 2 (USD)</t>
         </is>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="13">
         <f>B11-B14</f>
         <v/>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="13">
         <f>C11-C14</f>
         <v/>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="13">
         <f>D11-D14</f>
         <v/>
       </c>
@@ -3153,15 +3163,15 @@
           <t>EBITDA Ano 3 (USD)</t>
         </is>
       </c>
-      <c r="B18" s="14">
+      <c r="B18" s="13">
         <f>B12-B15</f>
         <v/>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="13">
         <f>C12-C15</f>
         <v/>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="13">
         <f>D12-D15</f>
         <v/>
       </c>
@@ -3172,15 +3182,15 @@
           <t>Inversion inicial (USD)</t>
         </is>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="13">
         <f>'Inversion y OPEX'!$C$8</f>
         <v/>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="13">
         <f>'Inversion y OPEX'!$C$8</f>
         <v/>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="13">
         <f>'Inversion y OPEX'!$C$8</f>
         <v/>
       </c>
@@ -3213,15 +3223,15 @@
           <t>EBITDA acumulado 3 anios</t>
         </is>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="13">
         <f>SUM(B16:B18)</f>
         <v/>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <f>SUM(C16:C18)</f>
         <v/>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="13">
         <f>SUM(D16:D18)</f>
         <v/>
       </c>
@@ -3232,15 +3242,15 @@
           <t>ROI 3 anios (%)</t>
         </is>
       </c>
-      <c r="B23" s="17">
+      <c r="B23" s="16">
         <f>(B22-B19)/B19</f>
         <v/>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="16">
         <f>(C22-C19)/C19</f>
         <v/>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="16">
         <f>(D22-D19)/D19</f>
         <v/>
       </c>
@@ -3251,15 +3261,15 @@
           <t>VPN (USD)</t>
         </is>
       </c>
-      <c r="B24" s="14">
+      <c r="B24" s="13">
         <f>-B19 + B16/(1+$E$2) + B17/(1+$E$2)^2 + B18/(1+$E$2)^3</f>
         <v/>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="13">
         <f>-C19 + C16/(1+$E$2) + C17/(1+$E$2)^2 + C18/(1+$E$2)^3</f>
         <v/>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="13">
         <f>-D19 + D16/(1+$E$2) + D17/(1+$E$2)^2 + D18/(1+$E$2)^3</f>
         <v/>
       </c>
@@ -3270,15 +3280,15 @@
           <t>TIR (%)</t>
         </is>
       </c>
-      <c r="B25" s="17">
+      <c r="B25" s="16">
         <f>IRR(B28:B31)</f>
         <v/>
       </c>
-      <c r="C25" s="17">
+      <c r="C25" s="16">
         <f>IRR(C28:C31)</f>
         <v/>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="16">
         <f>IRR(D28:D31)</f>
         <v/>
       </c>
@@ -3289,15 +3299,15 @@
           <t>Payback simple (meses, base EBITDA Ano 1)</t>
         </is>
       </c>
-      <c r="B26" s="18">
+      <c r="B26" s="17">
         <f>B19/(B16/12)</f>
         <v/>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="17">
         <f>C19/(C16/12)</f>
         <v/>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="17">
         <f>D19/(D16/12)</f>
         <v/>
       </c>
@@ -3308,15 +3318,15 @@
           <t>Flujo 0 (=-inversion)</t>
         </is>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="13">
         <f>-B19</f>
         <v/>
       </c>
-      <c r="C28" s="14">
+      <c r="C28" s="13">
         <f>-C19</f>
         <v/>
       </c>
-      <c r="D28" s="14">
+      <c r="D28" s="13">
         <f>-D19</f>
         <v/>
       </c>
@@ -3327,15 +3337,15 @@
           <t>Flujo Ano 1</t>
         </is>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="13">
         <f>B16</f>
         <v/>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="13">
         <f>C16</f>
         <v/>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="13">
         <f>D16</f>
         <v/>
       </c>
@@ -3346,15 +3356,15 @@
           <t>Flujo Ano 2</t>
         </is>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="13">
         <f>B17</f>
         <v/>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="13">
         <f>C17</f>
         <v/>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="13">
         <f>D17</f>
         <v/>
       </c>
@@ -3365,21 +3375,21 @@
           <t>Flujo Ano 3</t>
         </is>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="13">
         <f>B18</f>
         <v/>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="13">
         <f>C18</f>
         <v/>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="13">
         <f>D18</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>Nota: ROI = (EBITDA acumulado - inversion)/inversion. VPN descuenta los EBITDA anuales a la tasa editable (E2). TIR via IRR sobre flujos anuales (filas 28-31). El Payback simple usa el EBITDA mensual del Ano 1 (metodo conservador/lineal); el payback real considerando el crecimiento de los Anos 2-3 es menor (ver documento de analisis). Cambia ARPU, cuentas o la tasa y todo recalcula.</t>
         </is>

</xml_diff>